<commit_message>
Se agrega cambios para carga masiva- se queda estable
</commit_message>
<xml_diff>
--- a/backend/uploads/plantilla_clientes.xlsx
+++ b/backend/uploads/plantilla_clientes.xlsx
@@ -452,10 +452,10 @@
         <v>Juan Pérez García</v>
       </c>
       <c r="B2" t="str">
-        <v>961-123-4567</v>
+        <v>9611234567</v>
       </c>
       <c r="C2" t="str">
-        <v>961-123-4568</v>
+        <v>9611234568</v>
       </c>
       <c r="D2" t="str">
         <v>juan.perez@email.com</v>
@@ -470,7 +470,7 @@
         <v>PEGJ850315ABC</v>
       </c>
       <c r="H2" t="str">
-        <v>612 - Personas Físicas con Actividades Empresariales</v>
+        <v>612</v>
       </c>
       <c r="I2" t="str">
         <v>Av. Central 123, Col. Centro, Tuxtla Gutiérrez, Chiapas</v>
@@ -479,7 +479,7 @@
         <v>29000</v>
       </c>
       <c r="K2" t="str">
-        <v>G03 - Gastos en general</v>
+        <v>G03</v>
       </c>
     </row>
     <row r="3">
@@ -487,13 +487,13 @@
         <v>Comercializadora López S.A. de C.V.</v>
       </c>
       <c r="B3" t="str">
-        <v>961-234-5678</v>
+        <v>9612345678</v>
       </c>
       <c r="C3" t="str">
         <v/>
       </c>
       <c r="D3" t="str">
-        <v>contacto@lopez.com.mx</v>
+        <v/>
       </c>
       <c r="E3" t="str">
         <v>Blvd. Belisario Domínguez 456, Col. Moctezuma, Tuxtla Gutiérrez, Chiapas</v>
@@ -505,7 +505,7 @@
         <v>CLS920810XYZ</v>
       </c>
       <c r="H3" t="str">
-        <v>601 - General de Ley Personas Morales</v>
+        <v>601</v>
       </c>
       <c r="I3" t="str">
         <v>Blvd. Belisario Domínguez 456, Col. Moctezuma, Tuxtla Gutiérrez, Chiapas</v>
@@ -514,7 +514,7 @@
         <v>29030</v>
       </c>
       <c r="K3" t="str">
-        <v>G01 - Adquisición de mercancías</v>
+        <v>G01</v>
       </c>
     </row>
     <row r="4">
@@ -522,10 +522,10 @@
         <v>María González Hernández</v>
       </c>
       <c r="B4" t="str">
-        <v>967-345-6789</v>
+        <v>9673456789</v>
       </c>
       <c r="C4" t="str">
-        <v>967-345-6790</v>
+        <v>9673456790</v>
       </c>
       <c r="D4" t="str">
         <v>maria.gonzalez@email.com</v>
@@ -540,7 +540,7 @@
         <v>GOHM750425DEF</v>
       </c>
       <c r="H4" t="str">
-        <v>612 - Personas Físicas con Actividades Empresariales</v>
+        <v>612</v>
       </c>
       <c r="I4" t="str">
         <v>Real de Guadalupe 789, Centro, San Cristóbal de las Casas, Chiapas</v>
@@ -549,7 +549,7 @@
         <v>29200</v>
       </c>
       <c r="K4" t="str">
-        <v>G03 - Gastos en general</v>
+        <v>G03</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
se corrige id 1 y 3 de plan de trabajo
</commit_message>
<xml_diff>
--- a/backend/uploads/plantilla_clientes.xlsx
+++ b/backend/uploads/plantilla_clientes.xlsx
@@ -407,7 +407,7 @@
     <col min="6" max="6" width="30.83203125" customWidth="1"/>
     <col min="7" max="7" width="15.83203125" customWidth="1"/>
     <col min="8" max="8" width="40.83203125" customWidth="1"/>
-    <col min="9" max="9" width="40.83203125" customWidth="1"/>
+    <col min="9" max="9" width="50.83203125" customWidth="1"/>
     <col min="10" max="10" width="12.83203125" customWidth="1"/>
     <col min="11" max="11" width="35.83203125" customWidth="1"/>
   </cols>
@@ -438,7 +438,7 @@
         <v>regimen fiscal</v>
       </c>
       <c r="I1" t="str">
-        <v>direccion</v>
+        <v>direccion de facturacion</v>
       </c>
       <c r="J1" t="str">
         <v>codigo postal</v>
@@ -461,7 +461,7 @@
         <v>juan.perez@email.com</v>
       </c>
       <c r="E2" t="str">
-        <v>Av. Central 123, Col. Centro, Tuxtla Gutiérrez, Chiapas</v>
+        <v>Av. Central 123, Local 5, Col. Centro, Tuxtla Gutiérrez, Chiapas</v>
       </c>
       <c r="F2" t="str">
         <v>Juan Pérez García</v>
@@ -496,7 +496,7 @@
         <v/>
       </c>
       <c r="E3" t="str">
-        <v>Blvd. Belisario Domínguez 456, Col. Moctezuma, Tuxtla Gutiérrez, Chiapas</v>
+        <v>Bodega 3, Parque Industrial, Tuxtla Gutiérrez, Chiapas</v>
       </c>
       <c r="F3" t="str">
         <v>Comercializadora López S.A. de C.V.</v>

</xml_diff>